<commit_message>
updated the print cmf coordinates and uses the new cmf template
</commit_message>
<xml_diff>
--- a/core/main/templates/print_excel/new_cmf_template.xlsx
+++ b/core/main/templates/print_excel/new_cmf_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brant\VS Code Web\ColorMatch\core\main\templates\print_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A927A3A9-547B-4F68-82AA-6013750613D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74221F3A-685B-41C2-8974-93296B0B82EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{A6AD9F22-8F09-456A-8FB6-C96A1D80AD5A}"/>
+    <workbookView xWindow="3120" yWindow="930" windowWidth="16395" windowHeight="15270" xr2:uid="{A6AD9F22-8F09-456A-8FB6-C96A1D80AD5A}"/>
   </bookViews>
   <sheets>
     <sheet name="REVISE CMF 02-FINAL" sheetId="1" r:id="rId1"/>
@@ -298,7 +298,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -339,22 +338,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -364,18 +354,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -387,6 +378,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1384,100 +1384,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="26"/>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="26"/>
+      <c r="A1" s="22"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="26"/>
-      <c r="L2" s="26"/>
-      <c r="M2" s="26"/>
-      <c r="N2" s="26"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="26"/>
+      <c r="A2" s="22"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
     </row>
     <row r="3" spans="1:16" ht="21" x14ac:dyDescent="0.35">
-      <c r="A3" s="26"/>
-      <c r="B3" s="26"/>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="27" t="s">
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="M3" s="27"/>
-      <c r="N3" s="27"/>
-      <c r="O3" s="27"/>
-      <c r="P3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="22"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="26"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="26"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="26"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
     </row>
     <row r="6" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
-      <c r="B6" s="26"/>
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
       <c r="C6" s="2" t="s">
         <v>50</v>
       </c>
@@ -1485,21 +1485,21 @@
       <c r="E6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="23"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="26"/>
-      <c r="M6" s="26"/>
-      <c r="N6" s="26"/>
-      <c r="O6" s="26"/>
-      <c r="P6" s="26"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="18"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
     </row>
     <row r="7" spans="1:16" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="26"/>
-      <c r="B7" s="26"/>
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -1513,11 +1513,11 @@
       <c r="M7" s="1"/>
       <c r="N7" s="1"/>
       <c r="O7" s="1"/>
-      <c r="P7" s="26"/>
+      <c r="P7" s="22"/>
     </row>
     <row r="8" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="26"/>
-      <c r="B8" s="26"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="22"/>
       <c r="C8" s="2" t="s">
         <v>49</v>
       </c>
@@ -1525,21 +1525,21 @@
       <c r="E8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
-      <c r="P8" s="26"/>
+      <c r="P8" s="22"/>
     </row>
     <row r="9" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="26"/>
-      <c r="B9" s="26"/>
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -1553,11 +1553,11 @@
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
-      <c r="P9" s="26"/>
+      <c r="P9" s="22"/>
     </row>
     <row r="10" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
       <c r="C10" s="2" t="s">
         <v>48</v>
       </c>
@@ -1565,29 +1565,29 @@
       <c r="E10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="29"/>
-      <c r="J10" s="29"/>
-      <c r="P10" s="26"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24"/>
+      <c r="I10" s="24"/>
+      <c r="J10" s="24"/>
+      <c r="P10" s="22"/>
     </row>
     <row r="11" spans="1:16" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="26"/>
-      <c r="B11" s="26"/>
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="19"/>
-      <c r="J11" s="19"/>
-      <c r="P11" s="26"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="P11" s="22"/>
     </row>
     <row r="12" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
       <c r="C12" s="2" t="s">
         <v>47</v>
       </c>
@@ -1595,29 +1595,29 @@
       <c r="E12" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="29"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="29"/>
-      <c r="P12" s="26"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="P12" s="22"/>
     </row>
     <row r="13" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="26"/>
-      <c r="B13" s="26"/>
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="19"/>
-      <c r="J13" s="19"/>
-      <c r="P13" s="26"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="P13" s="22"/>
     </row>
     <row r="14" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26"/>
-      <c r="B14" s="26"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
       <c r="C14" s="2" t="s">
         <v>46</v>
       </c>
@@ -1625,20 +1625,20 @@
       <c r="E14" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
       <c r="K14" s="2"/>
       <c r="L14" s="2"/>
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
-      <c r="P14" s="26"/>
+      <c r="P14" s="22"/>
     </row>
     <row r="15" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="26"/>
-      <c r="B15" s="26"/>
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -1647,11 +1647,11 @@
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
-      <c r="P15" s="26"/>
+      <c r="P15" s="22"/>
     </row>
     <row r="16" spans="1:16" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
       <c r="C16" s="2" t="s">
         <v>45</v>
       </c>
@@ -1659,19 +1659,19 @@
       <c r="E16" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F16" s="4"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I16" s="4"/>
+      <c r="I16" s="3"/>
       <c r="J16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="P16" s="26"/>
+      <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -1685,11 +1685,11 @@
       <c r="M17" s="2"/>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
-      <c r="P17" s="26"/>
+      <c r="P17" s="22"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="26"/>
-      <c r="B18" s="26"/>
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
       <c r="C18" s="2" t="s">
         <v>42</v>
       </c>
@@ -1697,40 +1697,40 @@
       <c r="E18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F18" s="14"/>
+      <c r="F18" s="13"/>
       <c r="G18" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H18" s="5"/>
-      <c r="L18" s="14"/>
+      <c r="H18" s="4"/>
+      <c r="L18" s="13"/>
       <c r="M18" s="2" t="s">
         <v>40</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
-      <c r="P18" s="26"/>
+      <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="26"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="26"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
-      <c r="P19" s="26"/>
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="22"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
     </row>
     <row r="20" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="26"/>
-      <c r="B20" s="26"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
       <c r="C20" s="2" t="s">
         <v>39</v>
       </c>
@@ -1738,21 +1738,21 @@
       <c r="E20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="1"/>
       <c r="N20" s="1"/>
       <c r="O20" s="1"/>
-      <c r="P20" s="26"/>
+      <c r="P20" s="22"/>
     </row>
     <row r="21" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="26"/>
-      <c r="B21" s="26"/>
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -1766,11 +1766,11 @@
       <c r="M21" s="1"/>
       <c r="N21" s="1"/>
       <c r="O21" s="1"/>
-      <c r="P21" s="26"/>
+      <c r="P21" s="22"/>
     </row>
     <row r="22" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="26"/>
-      <c r="B22" s="26"/>
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="2" t="s">
         <v>38</v>
       </c>
@@ -1778,21 +1778,21 @@
       <c r="E22" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="29"/>
-      <c r="G22" s="29"/>
-      <c r="H22" s="29"/>
-      <c r="I22" s="29"/>
-      <c r="J22" s="29"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="24"/>
+      <c r="I22" s="24"/>
+      <c r="J22" s="24"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
       <c r="M22" s="1"/>
       <c r="N22" s="1"/>
       <c r="O22" s="1"/>
-      <c r="P22" s="26"/>
+      <c r="P22" s="22"/>
     </row>
     <row r="23" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26"/>
+      <c r="A23" s="22"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -1806,11 +1806,11 @@
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
       <c r="O23" s="1"/>
-      <c r="P23" s="26"/>
+      <c r="P23" s="22"/>
     </row>
     <row r="24" spans="1:16" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="26"/>
-      <c r="B24" s="26"/>
+      <c r="A24" s="22"/>
+      <c r="B24" s="22"/>
       <c r="C24" s="2" t="s">
         <v>37</v>
       </c>
@@ -1818,94 +1818,94 @@
       <c r="E24" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F24" s="18"/>
+      <c r="F24" s="3"/>
       <c r="G24" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="I24" s="18"/>
+      <c r="I24" s="3"/>
       <c r="J24" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="L24" s="4"/>
+      <c r="L24" s="3"/>
       <c r="M24" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="P24" s="26"/>
+      <c r="P24" s="22"/>
     </row>
     <row r="25" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="26"/>
-      <c r="B25" s="26"/>
-      <c r="C25" s="26"/>
-      <c r="D25" s="26"/>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26"/>
-      <c r="G25" s="26"/>
-      <c r="H25" s="26"/>
-      <c r="I25" s="26"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="26"/>
-      <c r="L25" s="26"/>
-      <c r="M25" s="26"/>
-      <c r="N25" s="26"/>
-      <c r="O25" s="26"/>
-      <c r="P25" s="26"/>
+      <c r="A25" s="22"/>
+      <c r="B25" s="22"/>
+      <c r="C25" s="22"/>
+      <c r="D25" s="22"/>
+      <c r="E25" s="22"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="22"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="22"/>
+      <c r="O25" s="22"/>
+      <c r="P25" s="22"/>
     </row>
     <row r="26" spans="1:16" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="26"/>
-      <c r="B26" s="26"/>
-      <c r="F26" s="4"/>
+      <c r="A26" s="22"/>
+      <c r="B26" s="22"/>
+      <c r="F26" s="3"/>
       <c r="G26" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="I26" s="4"/>
+      <c r="I26" s="3"/>
       <c r="J26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="L26" s="4"/>
+      <c r="L26" s="3"/>
       <c r="M26" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="P26" s="26"/>
+      <c r="P26" s="22"/>
     </row>
     <row r="27" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="26"/>
-      <c r="B27" s="26"/>
-      <c r="F27" s="6"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="F27" s="5"/>
       <c r="G27" s="2"/>
-      <c r="I27" s="6"/>
+      <c r="I27" s="5"/>
       <c r="J27" s="2"/>
-      <c r="L27" s="6"/>
+      <c r="L27" s="5"/>
       <c r="M27" s="2"/>
-      <c r="P27" s="26"/>
+      <c r="P27" s="22"/>
     </row>
     <row r="28" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="26"/>
-      <c r="B28" s="26"/>
-      <c r="F28" s="4"/>
+      <c r="A28" s="22"/>
+      <c r="B28" s="22"/>
+      <c r="F28" s="3"/>
       <c r="G28" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H28" s="7"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="6"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+      <c r="J28" s="25"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="5"/>
       <c r="M28" s="2"/>
-      <c r="P28" s="26"/>
+      <c r="P28" s="22"/>
     </row>
     <row r="29" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
-      <c r="F29" s="6"/>
-      <c r="I29" s="6"/>
+      <c r="A29" s="22"/>
+      <c r="B29" s="22"/>
+      <c r="F29" s="5"/>
+      <c r="I29" s="5"/>
       <c r="J29" s="2"/>
-      <c r="L29" s="6"/>
+      <c r="L29" s="5"/>
       <c r="M29" s="2"/>
-      <c r="P29" s="26"/>
+      <c r="P29" s="22"/>
     </row>
     <row r="30" spans="1:16" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="26"/>
-      <c r="B30" s="26"/>
+      <c r="A30" s="22"/>
+      <c r="B30" s="22"/>
       <c r="C30" s="2" t="s">
         <v>30</v>
       </c>
@@ -1913,11 +1913,11 @@
       <c r="E30" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F30" s="4"/>
+      <c r="F30" s="3"/>
       <c r="G30" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I30" s="4"/>
+      <c r="I30" s="3"/>
       <c r="J30" s="2" t="s">
         <v>4</v>
       </c>
@@ -1926,22 +1926,22 @@
       <c r="M30" s="1"/>
       <c r="N30" s="1"/>
       <c r="O30" s="1"/>
-      <c r="P30" s="26"/>
+      <c r="P30" s="22"/>
     </row>
     <row r="31" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-      <c r="J31" s="30"/>
-      <c r="K31" s="30"/>
-      <c r="L31" s="30"/>
-      <c r="M31" s="30"/>
-      <c r="P31" s="26"/>
+      <c r="A31" s="22"/>
+      <c r="B31" s="22"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="P31" s="22"/>
     </row>
     <row r="32" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
+      <c r="A32" s="22"/>
+      <c r="B32" s="22"/>
       <c r="C32" s="2" t="s">
         <v>29</v>
       </c>
@@ -1949,92 +1949,92 @@
       <c r="E32" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F32" s="4"/>
+      <c r="F32" s="3"/>
       <c r="G32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="I32" s="4"/>
+      <c r="I32" s="3"/>
       <c r="J32" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L32" s="4"/>
+      <c r="L32" s="3"/>
       <c r="M32" s="2" t="s">
         <v>26</v>
       </c>
       <c r="N32" s="2"/>
-      <c r="O32" s="7"/>
-      <c r="P32" s="26"/>
+      <c r="O32" s="6"/>
+      <c r="P32" s="22"/>
     </row>
     <row r="33" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="26"/>
-      <c r="B33" s="26"/>
+      <c r="A33" s="22"/>
+      <c r="B33" s="22"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
-      <c r="F33" s="6"/>
+      <c r="F33" s="5"/>
       <c r="G33" s="2"/>
-      <c r="I33" s="6"/>
+      <c r="I33" s="5"/>
       <c r="J33" s="2"/>
-      <c r="K33" s="6"/>
+      <c r="K33" s="5"/>
       <c r="L33" s="2"/>
       <c r="N33" s="2"/>
-      <c r="P33" s="26"/>
+      <c r="P33" s="22"/>
     </row>
     <row r="34" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="26"/>
-      <c r="B34" s="26"/>
-      <c r="C34" s="8" t="s">
+      <c r="A34" s="22"/>
+      <c r="B34" s="22"/>
+      <c r="C34" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8" t="s">
+      <c r="D34" s="7"/>
+      <c r="E34" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F34" s="21"/>
-      <c r="G34" s="21"/>
-      <c r="H34" s="21"/>
-      <c r="I34" s="21"/>
-      <c r="J34" s="21"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="34"/>
+      <c r="J34" s="34"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
       <c r="N34" s="1"/>
       <c r="O34" s="1"/>
-      <c r="P34" s="26"/>
+      <c r="P34" s="22"/>
     </row>
     <row r="35" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="26"/>
-      <c r="B35" s="26"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="9"/>
-      <c r="G35" s="9"/>
-      <c r="H35" s="9"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
+      <c r="A35" s="22"/>
+      <c r="B35" s="22"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="33"/>
+      <c r="G35" s="33"/>
+      <c r="H35" s="33"/>
+      <c r="I35" s="33"/>
+      <c r="J35" s="33"/>
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
       <c r="N35" s="1"/>
       <c r="O35" s="1"/>
-      <c r="P35" s="26"/>
+      <c r="P35" s="22"/>
     </row>
     <row r="36" spans="1:16" ht="16.350000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="26"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="8" t="s">
+      <c r="A36" s="22"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8" t="s">
+      <c r="D36" s="7"/>
+      <c r="E36" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F36" s="21"/>
-      <c r="G36" s="21"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="21"/>
+      <c r="F36" s="34"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="34"/>
+      <c r="J36" s="34"/>
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -2042,15 +2042,15 @@
       <c r="O36" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="P36" s="26"/>
+      <c r="P36" s="22"/>
     </row>
     <row r="37" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="26"/>
-      <c r="B37" s="26"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="9"/>
+      <c r="A37" s="22"/>
+      <c r="B37" s="22"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="8"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
@@ -2060,127 +2060,127 @@
       <c r="M37" s="1"/>
       <c r="N37" s="1"/>
       <c r="O37" s="1"/>
-      <c r="P37" s="26"/>
+      <c r="P37" s="22"/>
     </row>
     <row r="38" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="26"/>
-      <c r="B38" s="26"/>
-      <c r="C38" s="10" t="s">
+      <c r="A38" s="22"/>
+      <c r="B38" s="22"/>
+      <c r="C38" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D38" s="10"/>
-      <c r="E38" s="10" t="s">
+      <c r="D38" s="9"/>
+      <c r="E38" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F38" s="25"/>
-      <c r="G38" s="25"/>
-      <c r="H38" s="25"/>
-      <c r="I38" s="25"/>
-      <c r="J38" s="25"/>
-      <c r="K38" s="26"/>
-      <c r="L38" s="26"/>
-      <c r="M38" s="26"/>
-      <c r="N38" s="26"/>
-      <c r="O38" s="26"/>
-      <c r="P38" s="26"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="21"/>
+      <c r="H38" s="21"/>
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="22"/>
+      <c r="L38" s="22"/>
+      <c r="M38" s="22"/>
+      <c r="N38" s="22"/>
+      <c r="O38" s="22"/>
+      <c r="P38" s="22"/>
     </row>
     <row r="39" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="26"/>
-      <c r="B39" s="26"/>
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
-      <c r="G39" s="26"/>
-      <c r="H39" s="26"/>
-      <c r="I39" s="26"/>
-      <c r="J39" s="26"/>
-      <c r="K39" s="26"/>
-      <c r="L39" s="26"/>
-      <c r="M39" s="26"/>
-      <c r="N39" s="26"/>
-      <c r="O39" s="26"/>
-      <c r="P39" s="26"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="22"/>
+      <c r="I39" s="22"/>
+      <c r="J39" s="22"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="22"/>
+      <c r="M39" s="22"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
+      <c r="P39" s="22"/>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="26"/>
-      <c r="B40" s="26"/>
-      <c r="C40" s="10" t="s">
+      <c r="A40" s="22"/>
+      <c r="B40" s="22"/>
+      <c r="C40" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="10"/>
-      <c r="E40" s="10" t="s">
+      <c r="D40" s="9"/>
+      <c r="E40" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="F40" s="4"/>
+      <c r="F40" s="3"/>
       <c r="G40" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I40" s="4"/>
+      <c r="I40" s="3"/>
       <c r="J40" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="L40" s="4"/>
+      <c r="L40" s="3"/>
       <c r="M40" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="N40" s="26"/>
-      <c r="O40" s="26"/>
-      <c r="P40" s="26"/>
+      <c r="N40" s="22"/>
+      <c r="O40" s="22"/>
+      <c r="P40" s="22"/>
     </row>
     <row r="41" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="26"/>
-      <c r="B41" s="26"/>
-      <c r="C41" s="26"/>
-      <c r="D41" s="26"/>
-      <c r="E41" s="26"/>
-      <c r="F41" s="26"/>
-      <c r="G41" s="26"/>
-      <c r="H41" s="26"/>
-      <c r="I41" s="26"/>
-      <c r="J41" s="26"/>
-      <c r="K41" s="26"/>
-      <c r="L41" s="26"/>
-      <c r="M41" s="26"/>
-      <c r="N41" s="26"/>
-      <c r="O41" s="26"/>
-      <c r="P41" s="26"/>
+      <c r="A41" s="22"/>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="22"/>
+      <c r="K41" s="22"/>
+      <c r="L41" s="22"/>
+      <c r="M41" s="22"/>
+      <c r="N41" s="22"/>
+      <c r="O41" s="22"/>
+      <c r="P41" s="22"/>
     </row>
     <row r="42" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="26"/>
-      <c r="B42" s="26"/>
-      <c r="F42" s="4"/>
+      <c r="A42" s="22"/>
+      <c r="B42" s="22"/>
+      <c r="F42" s="3"/>
       <c r="G42" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="I42" s="4"/>
+      <c r="I42" s="3"/>
       <c r="J42" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K42" s="3"/>
-      <c r="L42" s="3"/>
-      <c r="M42" s="3"/>
-      <c r="N42" s="3"/>
-      <c r="P42" s="26"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="18"/>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
+      <c r="P42" s="22"/>
     </row>
     <row r="43" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="26"/>
-      <c r="B43" s="26"/>
-      <c r="F43" s="26"/>
-      <c r="G43" s="26"/>
-      <c r="H43" s="26"/>
-      <c r="I43" s="26"/>
-      <c r="J43" s="26"/>
-      <c r="K43" s="26"/>
-      <c r="L43" s="26"/>
-      <c r="M43" s="26"/>
-      <c r="N43" s="26"/>
-      <c r="O43" s="26"/>
-      <c r="P43" s="26"/>
+      <c r="A43" s="22"/>
+      <c r="B43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="22"/>
+      <c r="J43" s="22"/>
+      <c r="K43" s="22"/>
+      <c r="L43" s="22"/>
+      <c r="M43" s="22"/>
+      <c r="N43" s="22"/>
+      <c r="O43" s="22"/>
+      <c r="P43" s="22"/>
     </row>
     <row r="44" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="26"/>
-      <c r="B44" s="26"/>
+      <c r="A44" s="22"/>
+      <c r="B44" s="22"/>
       <c r="C44" s="2" t="s">
         <v>17</v>
       </c>
@@ -2188,39 +2188,39 @@
       <c r="E44" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F44" s="25"/>
-      <c r="G44" s="25"/>
-      <c r="H44" s="25"/>
-      <c r="I44" s="25"/>
-      <c r="J44" s="25"/>
-      <c r="K44" s="11"/>
-      <c r="L44" s="12"/>
-      <c r="M44" s="12"/>
-      <c r="N44" s="12"/>
-      <c r="O44" s="12"/>
-      <c r="P44" s="26"/>
+      <c r="F44" s="32"/>
+      <c r="G44" s="32"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="32"/>
+      <c r="J44" s="32"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="11"/>
+      <c r="M44" s="11"/>
+      <c r="N44" s="11"/>
+      <c r="O44" s="11"/>
+      <c r="P44" s="22"/>
     </row>
     <row r="45" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="26"/>
-      <c r="B45" s="26"/>
+      <c r="A45" s="22"/>
+      <c r="B45" s="22"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="8"/>
-      <c r="I45" s="8"/>
-      <c r="J45" s="8"/>
-      <c r="K45" s="11"/>
-      <c r="L45" s="12"/>
-      <c r="M45" s="12"/>
-      <c r="N45" s="12"/>
-      <c r="O45" s="12"/>
-      <c r="P45" s="26"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="7"/>
+      <c r="I45" s="7"/>
+      <c r="J45" s="7"/>
+      <c r="K45" s="10"/>
+      <c r="L45" s="11"/>
+      <c r="M45" s="11"/>
+      <c r="N45" s="11"/>
+      <c r="O45" s="11"/>
+      <c r="P45" s="22"/>
     </row>
     <row r="46" spans="1:16" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="26"/>
-      <c r="B46" s="26"/>
+      <c r="A46" s="22"/>
+      <c r="B46" s="22"/>
       <c r="C46" s="2" t="s">
         <v>16</v>
       </c>
@@ -2228,43 +2228,43 @@
       <c r="E46" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F46" s="4"/>
+      <c r="F46" s="3"/>
       <c r="G46" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I46" s="4"/>
+      <c r="I46" s="3"/>
       <c r="J46" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K46" s="31" t="s">
+      <c r="K46" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="L46" s="31"/>
-      <c r="M46" s="31"/>
-      <c r="N46" s="31"/>
-      <c r="O46" s="31"/>
-      <c r="P46" s="26"/>
+      <c r="L46" s="28"/>
+      <c r="M46" s="28"/>
+      <c r="N46" s="28"/>
+      <c r="O46" s="28"/>
+      <c r="P46" s="22"/>
     </row>
     <row r="47" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="26"/>
-      <c r="B47" s="26"/>
+      <c r="A47" s="22"/>
+      <c r="B47" s="22"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
-      <c r="F47" s="6"/>
+      <c r="F47" s="5"/>
       <c r="G47" s="2"/>
-      <c r="I47" s="6"/>
+      <c r="I47" s="5"/>
       <c r="J47" s="2"/>
-      <c r="K47" s="31"/>
-      <c r="L47" s="31"/>
-      <c r="M47" s="31"/>
-      <c r="N47" s="31"/>
-      <c r="O47" s="31"/>
-      <c r="P47" s="26"/>
+      <c r="K47" s="28"/>
+      <c r="L47" s="28"/>
+      <c r="M47" s="28"/>
+      <c r="N47" s="28"/>
+      <c r="O47" s="28"/>
+      <c r="P47" s="22"/>
     </row>
     <row r="48" spans="1:16" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="26"/>
-      <c r="B48" s="26"/>
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
       <c r="C48" s="2" t="s">
         <v>14</v>
       </c>
@@ -2272,39 +2272,39 @@
       <c r="E48" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F48" s="25"/>
-      <c r="G48" s="25"/>
-      <c r="H48" s="25"/>
-      <c r="I48" s="25"/>
-      <c r="J48" s="25"/>
-      <c r="K48" s="31"/>
-      <c r="L48" s="31"/>
-      <c r="M48" s="31"/>
-      <c r="N48" s="31"/>
-      <c r="O48" s="31"/>
-      <c r="P48" s="26"/>
+      <c r="F48" s="32"/>
+      <c r="G48" s="32"/>
+      <c r="H48" s="32"/>
+      <c r="I48" s="32"/>
+      <c r="J48" s="32"/>
+      <c r="K48" s="28"/>
+      <c r="L48" s="28"/>
+      <c r="M48" s="28"/>
+      <c r="N48" s="28"/>
+      <c r="O48" s="28"/>
+      <c r="P48" s="22"/>
     </row>
     <row r="49" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="26"/>
-      <c r="B49" s="26"/>
+      <c r="A49" s="22"/>
+      <c r="B49" s="22"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="8"/>
-      <c r="I49" s="8"/>
-      <c r="J49" s="8"/>
-      <c r="K49" s="31"/>
-      <c r="L49" s="31"/>
-      <c r="M49" s="31"/>
-      <c r="N49" s="31"/>
-      <c r="O49" s="31"/>
-      <c r="P49" s="26"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="7"/>
+      <c r="I49" s="7"/>
+      <c r="J49" s="7"/>
+      <c r="K49" s="28"/>
+      <c r="L49" s="28"/>
+      <c r="M49" s="28"/>
+      <c r="N49" s="28"/>
+      <c r="O49" s="28"/>
+      <c r="P49" s="22"/>
     </row>
     <row r="50" spans="1:16" ht="16.350000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="26"/>
-      <c r="B50" s="26"/>
+      <c r="A50" s="22"/>
+      <c r="B50" s="22"/>
       <c r="C50" s="2" t="s">
         <v>13</v>
       </c>
@@ -2312,42 +2312,42 @@
       <c r="E50" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F50" s="4"/>
+      <c r="F50" s="3"/>
       <c r="G50" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="I50" s="4"/>
+      <c r="I50" s="3"/>
       <c r="J50" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K50" s="31"/>
-      <c r="L50" s="31"/>
-      <c r="M50" s="31"/>
-      <c r="N50" s="31"/>
-      <c r="O50" s="31"/>
-      <c r="P50" s="26"/>
+      <c r="K50" s="28"/>
+      <c r="L50" s="28"/>
+      <c r="M50" s="28"/>
+      <c r="N50" s="28"/>
+      <c r="O50" s="28"/>
+      <c r="P50" s="22"/>
     </row>
     <row r="51" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="26"/>
-      <c r="B51" s="26"/>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
-      <c r="G51" s="26"/>
-      <c r="H51" s="26"/>
-      <c r="I51" s="26"/>
-      <c r="J51" s="26"/>
-      <c r="K51" s="26"/>
-      <c r="L51" s="26"/>
-      <c r="M51" s="26"/>
-      <c r="N51" s="26"/>
-      <c r="O51" s="26"/>
-      <c r="P51" s="26"/>
+      <c r="A51" s="22"/>
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
+      <c r="I51" s="22"/>
+      <c r="J51" s="22"/>
+      <c r="K51" s="22"/>
+      <c r="L51" s="22"/>
+      <c r="M51" s="22"/>
+      <c r="N51" s="22"/>
+      <c r="O51" s="22"/>
+      <c r="P51" s="22"/>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A52" s="26"/>
-      <c r="B52" s="26"/>
+      <c r="A52" s="22"/>
+      <c r="B52" s="22"/>
       <c r="C52" s="2" t="s">
         <v>12</v>
       </c>
@@ -2355,19 +2355,19 @@
       <c r="E52" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F52" s="4"/>
+      <c r="F52" s="3"/>
       <c r="G52" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I52" s="4"/>
+      <c r="I52" s="3"/>
       <c r="J52" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="P52" s="26"/>
+      <c r="P52" s="22"/>
     </row>
     <row r="53" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="26"/>
-      <c r="B53" s="26"/>
+      <c r="A53" s="22"/>
+      <c r="B53" s="22"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
@@ -2376,48 +2376,48 @@
       <c r="J53" s="2"/>
       <c r="M53" s="2"/>
       <c r="O53" s="2"/>
-      <c r="P53" s="26"/>
+      <c r="P53" s="22"/>
     </row>
     <row r="54" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="26"/>
-      <c r="B54" s="26"/>
+      <c r="A54" s="22"/>
+      <c r="B54" s="22"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
-      <c r="F54" s="4"/>
+      <c r="F54" s="3"/>
       <c r="G54" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H54" s="32"/>
-      <c r="I54" s="32"/>
-      <c r="J54" s="32"/>
-      <c r="K54" s="32"/>
-      <c r="L54" s="32"/>
+      <c r="H54" s="29"/>
+      <c r="I54" s="29"/>
+      <c r="J54" s="29"/>
+      <c r="K54" s="29"/>
+      <c r="L54" s="29"/>
       <c r="M54" s="2"/>
       <c r="O54" s="2"/>
-      <c r="P54" s="26"/>
+      <c r="P54" s="22"/>
     </row>
     <row r="55" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="26"/>
-      <c r="B55" s="26"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
-      <c r="G55" s="26"/>
-      <c r="H55" s="26"/>
-      <c r="I55" s="26"/>
-      <c r="J55" s="26"/>
-      <c r="K55" s="26"/>
-      <c r="L55" s="26"/>
-      <c r="M55" s="26"/>
-      <c r="N55" s="26"/>
-      <c r="O55" s="26"/>
-      <c r="P55" s="26"/>
+      <c r="A55" s="22"/>
+      <c r="B55" s="22"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="22"/>
+      <c r="H55" s="22"/>
+      <c r="I55" s="22"/>
+      <c r="J55" s="22"/>
+      <c r="K55" s="22"/>
+      <c r="L55" s="22"/>
+      <c r="M55" s="22"/>
+      <c r="N55" s="22"/>
+      <c r="O55" s="22"/>
+      <c r="P55" s="22"/>
     </row>
     <row r="56" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="26"/>
-      <c r="B56" s="26"/>
+      <c r="A56" s="22"/>
+      <c r="B56" s="22"/>
       <c r="C56" s="2" t="s">
         <v>8</v>
       </c>
@@ -2425,39 +2425,39 @@
       <c r="E56" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F56" s="25"/>
-      <c r="G56" s="25"/>
-      <c r="H56" s="25"/>
-      <c r="I56" s="25"/>
-      <c r="J56" s="25"/>
-      <c r="K56" s="33"/>
-      <c r="L56" s="33"/>
-      <c r="M56" s="33"/>
-      <c r="N56" s="33"/>
-      <c r="O56" s="33"/>
-      <c r="P56" s="26"/>
+      <c r="F56" s="32"/>
+      <c r="G56" s="32"/>
+      <c r="H56" s="32"/>
+      <c r="I56" s="32"/>
+      <c r="J56" s="32"/>
+      <c r="K56" s="30"/>
+      <c r="L56" s="30"/>
+      <c r="M56" s="30"/>
+      <c r="N56" s="30"/>
+      <c r="O56" s="30"/>
+      <c r="P56" s="22"/>
     </row>
     <row r="57" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="26"/>
-      <c r="B57" s="26"/>
+      <c r="A57" s="22"/>
+      <c r="B57" s="22"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
-      <c r="F57" s="8"/>
-      <c r="G57" s="8"/>
-      <c r="H57" s="8"/>
-      <c r="I57" s="8"/>
-      <c r="J57" s="8"/>
-      <c r="K57" s="8"/>
-      <c r="L57" s="8"/>
-      <c r="M57" s="8"/>
-      <c r="N57" s="8"/>
-      <c r="O57" s="8"/>
-      <c r="P57" s="26"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
+      <c r="N57" s="7"/>
+      <c r="O57" s="7"/>
+      <c r="P57" s="22"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="26"/>
-      <c r="B58" s="26"/>
+      <c r="A58" s="22"/>
+      <c r="B58" s="22"/>
       <c r="C58" s="2" t="s">
         <v>7</v>
       </c>
@@ -2465,347 +2465,348 @@
       <c r="E58" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F58" s="4"/>
+      <c r="F58" s="3"/>
       <c r="G58" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H58" s="13"/>
-      <c r="I58" s="14"/>
+      <c r="H58" s="12"/>
+      <c r="I58" s="13"/>
       <c r="J58" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K58" s="13"/>
-      <c r="L58" s="13"/>
-      <c r="M58" s="13" t="s">
+      <c r="K58" s="12"/>
+      <c r="L58" s="12"/>
+      <c r="M58" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="N58" s="13"/>
-      <c r="O58" s="13"/>
-      <c r="P58" s="26"/>
+      <c r="N58" s="12"/>
+      <c r="O58" s="12"/>
+      <c r="P58" s="22"/>
     </row>
     <row r="59" spans="1:16" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="26"/>
-      <c r="B59" s="26"/>
+      <c r="A59" s="22"/>
+      <c r="B59" s="22"/>
       <c r="E59" s="2"/>
-      <c r="P59" s="26"/>
+      <c r="P59" s="22"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="26"/>
-      <c r="B60" s="26"/>
+      <c r="A60" s="22"/>
+      <c r="B60" s="22"/>
       <c r="C60" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D60" s="2"/>
-      <c r="E60" s="15"/>
-      <c r="F60" s="16"/>
-      <c r="G60" s="16"/>
-      <c r="H60" s="16"/>
-      <c r="I60" s="16"/>
-      <c r="J60" s="16"/>
-      <c r="K60" s="16"/>
-      <c r="L60" s="16"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="16"/>
-      <c r="O60" s="16"/>
-      <c r="P60" s="26"/>
+      <c r="E60" s="14"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="15"/>
+      <c r="K60" s="15"/>
+      <c r="L60" s="15"/>
+      <c r="M60" s="15"/>
+      <c r="N60" s="15"/>
+      <c r="O60" s="15"/>
+      <c r="P60" s="22"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A61" s="26"/>
-      <c r="B61" s="26"/>
-      <c r="C61" s="15" t="s">
+      <c r="A61" s="22"/>
+      <c r="B61" s="22"/>
+      <c r="C61" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D61" s="15"/>
-      <c r="E61" s="16"/>
-      <c r="F61" s="16"/>
-      <c r="G61" s="16"/>
-      <c r="H61" s="16"/>
-      <c r="I61" s="16"/>
-      <c r="J61" s="16"/>
-      <c r="K61" s="16"/>
-      <c r="L61" s="16"/>
-      <c r="M61" s="16"/>
-      <c r="N61" s="16"/>
-      <c r="O61" s="16"/>
-      <c r="P61" s="26"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
+      <c r="I61" s="15"/>
+      <c r="J61" s="15"/>
+      <c r="K61" s="15"/>
+      <c r="L61" s="15"/>
+      <c r="M61" s="15"/>
+      <c r="N61" s="15"/>
+      <c r="O61" s="15"/>
+      <c r="P61" s="22"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A62" s="26"/>
-      <c r="B62" s="26"/>
-      <c r="C62" s="16"/>
-      <c r="D62" s="16"/>
-      <c r="E62" s="16"/>
-      <c r="F62" s="16"/>
-      <c r="G62" s="16"/>
-      <c r="H62" s="16"/>
-      <c r="I62" s="16"/>
-      <c r="J62" s="16"/>
-      <c r="K62" s="16"/>
-      <c r="L62" s="16"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="16"/>
-      <c r="O62" s="16"/>
-      <c r="P62" s="26"/>
+      <c r="A62" s="22"/>
+      <c r="B62" s="22"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="15"/>
+      <c r="H62" s="15"/>
+      <c r="I62" s="15"/>
+      <c r="J62" s="15"/>
+      <c r="K62" s="15"/>
+      <c r="L62" s="15"/>
+      <c r="M62" s="15"/>
+      <c r="N62" s="15"/>
+      <c r="O62" s="15"/>
+      <c r="P62" s="22"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A63" s="26"/>
-      <c r="B63" s="26"/>
-      <c r="C63" s="24"/>
-      <c r="D63" s="24"/>
-      <c r="E63" s="24"/>
-      <c r="F63" s="24"/>
-      <c r="G63" s="24"/>
-      <c r="H63" s="24"/>
-      <c r="I63" s="24"/>
-      <c r="J63" s="24"/>
-      <c r="K63" s="24"/>
-      <c r="L63" s="24"/>
-      <c r="M63" s="24"/>
-      <c r="N63" s="24"/>
-      <c r="O63" s="16"/>
-      <c r="P63" s="26"/>
+      <c r="A63" s="22"/>
+      <c r="B63" s="22"/>
+      <c r="C63" s="20"/>
+      <c r="D63" s="20"/>
+      <c r="E63" s="20"/>
+      <c r="F63" s="20"/>
+      <c r="G63" s="20"/>
+      <c r="H63" s="20"/>
+      <c r="I63" s="20"/>
+      <c r="J63" s="20"/>
+      <c r="K63" s="20"/>
+      <c r="L63" s="20"/>
+      <c r="M63" s="20"/>
+      <c r="N63" s="20"/>
+      <c r="O63" s="15"/>
+      <c r="P63" s="22"/>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A64" s="26"/>
-      <c r="B64" s="26"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="24"/>
-      <c r="E64" s="24"/>
-      <c r="F64" s="24"/>
-      <c r="G64" s="24"/>
-      <c r="H64" s="24"/>
-      <c r="I64" s="24"/>
-      <c r="J64" s="24"/>
-      <c r="K64" s="24"/>
-      <c r="L64" s="24"/>
-      <c r="M64" s="24"/>
-      <c r="N64" s="24"/>
-      <c r="O64" s="16"/>
-      <c r="P64" s="26"/>
+      <c r="A64" s="22"/>
+      <c r="B64" s="22"/>
+      <c r="C64" s="20"/>
+      <c r="D64" s="20"/>
+      <c r="E64" s="20"/>
+      <c r="F64" s="20"/>
+      <c r="G64" s="20"/>
+      <c r="H64" s="20"/>
+      <c r="I64" s="20"/>
+      <c r="J64" s="20"/>
+      <c r="K64" s="20"/>
+      <c r="L64" s="20"/>
+      <c r="M64" s="20"/>
+      <c r="N64" s="20"/>
+      <c r="O64" s="15"/>
+      <c r="P64" s="22"/>
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A65" s="26"/>
-      <c r="B65" s="26"/>
-      <c r="C65" s="24"/>
-      <c r="D65" s="24"/>
-      <c r="E65" s="24"/>
-      <c r="F65" s="24"/>
-      <c r="G65" s="24"/>
-      <c r="H65" s="24"/>
-      <c r="I65" s="24"/>
-      <c r="J65" s="24"/>
-      <c r="K65" s="24"/>
-      <c r="L65" s="24"/>
-      <c r="M65" s="24"/>
-      <c r="N65" s="24"/>
-      <c r="O65" s="16"/>
-      <c r="P65" s="26"/>
+      <c r="A65" s="22"/>
+      <c r="B65" s="22"/>
+      <c r="C65" s="20"/>
+      <c r="D65" s="20"/>
+      <c r="E65" s="20"/>
+      <c r="F65" s="20"/>
+      <c r="G65" s="20"/>
+      <c r="H65" s="20"/>
+      <c r="I65" s="20"/>
+      <c r="J65" s="20"/>
+      <c r="K65" s="20"/>
+      <c r="L65" s="20"/>
+      <c r="M65" s="20"/>
+      <c r="N65" s="20"/>
+      <c r="O65" s="15"/>
+      <c r="P65" s="22"/>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A66" s="26"/>
-      <c r="B66" s="26"/>
-      <c r="C66" s="24"/>
-      <c r="D66" s="24"/>
-      <c r="E66" s="24"/>
-      <c r="F66" s="24"/>
-      <c r="G66" s="24"/>
-      <c r="H66" s="24"/>
-      <c r="I66" s="24"/>
-      <c r="J66" s="24"/>
-      <c r="K66" s="24"/>
-      <c r="L66" s="24"/>
-      <c r="M66" s="24"/>
-      <c r="N66" s="24"/>
-      <c r="O66" s="16"/>
-      <c r="P66" s="26"/>
+      <c r="A66" s="22"/>
+      <c r="B66" s="22"/>
+      <c r="C66" s="20"/>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="20"/>
+      <c r="L66" s="20"/>
+      <c r="M66" s="20"/>
+      <c r="N66" s="20"/>
+      <c r="O66" s="15"/>
+      <c r="P66" s="22"/>
     </row>
     <row r="67" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="26"/>
-      <c r="B67" s="26"/>
-      <c r="C67" s="24"/>
-      <c r="D67" s="24"/>
-      <c r="E67" s="24"/>
-      <c r="F67" s="24"/>
-      <c r="G67" s="24"/>
-      <c r="H67" s="24"/>
-      <c r="I67" s="24"/>
-      <c r="J67" s="24"/>
-      <c r="K67" s="24"/>
-      <c r="L67" s="24"/>
-      <c r="M67" s="24"/>
-      <c r="N67" s="24"/>
-      <c r="O67" s="16"/>
-      <c r="P67" s="26"/>
+      <c r="A67" s="22"/>
+      <c r="B67" s="22"/>
+      <c r="C67" s="20"/>
+      <c r="D67" s="20"/>
+      <c r="E67" s="20"/>
+      <c r="F67" s="20"/>
+      <c r="G67" s="20"/>
+      <c r="H67" s="20"/>
+      <c r="I67" s="20"/>
+      <c r="J67" s="20"/>
+      <c r="K67" s="20"/>
+      <c r="L67" s="20"/>
+      <c r="M67" s="20"/>
+      <c r="N67" s="20"/>
+      <c r="O67" s="15"/>
+      <c r="P67" s="22"/>
     </row>
     <row r="68" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="26"/>
-      <c r="B68" s="26"/>
-      <c r="C68" s="24"/>
-      <c r="D68" s="24"/>
-      <c r="E68" s="24"/>
-      <c r="F68" s="24"/>
-      <c r="G68" s="24"/>
-      <c r="H68" s="24"/>
-      <c r="I68" s="24"/>
-      <c r="J68" s="24"/>
-      <c r="K68" s="24"/>
-      <c r="L68" s="24"/>
-      <c r="M68" s="24"/>
-      <c r="N68" s="24"/>
-      <c r="O68" s="16"/>
-      <c r="P68" s="26"/>
+      <c r="A68" s="22"/>
+      <c r="B68" s="22"/>
+      <c r="C68" s="20"/>
+      <c r="D68" s="20"/>
+      <c r="E68" s="20"/>
+      <c r="F68" s="20"/>
+      <c r="G68" s="20"/>
+      <c r="H68" s="20"/>
+      <c r="I68" s="20"/>
+      <c r="J68" s="20"/>
+      <c r="K68" s="20"/>
+      <c r="L68" s="20"/>
+      <c r="M68" s="20"/>
+      <c r="N68" s="20"/>
+      <c r="O68" s="15"/>
+      <c r="P68" s="22"/>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A69" s="26"/>
-      <c r="B69" s="26"/>
-      <c r="C69" s="24"/>
-      <c r="D69" s="24"/>
-      <c r="E69" s="24"/>
-      <c r="F69" s="24"/>
-      <c r="G69" s="24"/>
-      <c r="H69" s="24"/>
-      <c r="I69" s="24"/>
-      <c r="J69" s="24"/>
-      <c r="K69" s="24"/>
-      <c r="L69" s="24"/>
-      <c r="M69" s="24"/>
-      <c r="N69" s="24"/>
-      <c r="O69" s="16"/>
-      <c r="P69" s="26"/>
+      <c r="A69" s="22"/>
+      <c r="B69" s="22"/>
+      <c r="C69" s="20"/>
+      <c r="D69" s="20"/>
+      <c r="E69" s="20"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="20"/>
+      <c r="L69" s="20"/>
+      <c r="M69" s="20"/>
+      <c r="N69" s="20"/>
+      <c r="O69" s="15"/>
+      <c r="P69" s="22"/>
     </row>
     <row r="70" spans="1:16" ht="8.4499999999999993" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="26"/>
-      <c r="B70" s="26"/>
-      <c r="C70" s="16"/>
-      <c r="D70" s="16"/>
-      <c r="E70" s="16"/>
-      <c r="F70" s="16"/>
-      <c r="G70" s="16"/>
-      <c r="H70" s="16"/>
-      <c r="I70" s="16"/>
-      <c r="J70" s="16"/>
-      <c r="K70" s="16"/>
-      <c r="L70" s="16"/>
-      <c r="M70" s="16"/>
-      <c r="N70" s="16"/>
-      <c r="O70" s="16"/>
-      <c r="P70" s="26"/>
+      <c r="A70" s="22"/>
+      <c r="B70" s="22"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="15"/>
+      <c r="E70" s="15"/>
+      <c r="F70" s="15"/>
+      <c r="G70" s="15"/>
+      <c r="H70" s="15"/>
+      <c r="I70" s="15"/>
+      <c r="J70" s="15"/>
+      <c r="K70" s="15"/>
+      <c r="L70" s="15"/>
+      <c r="M70" s="15"/>
+      <c r="N70" s="15"/>
+      <c r="O70" s="15"/>
+      <c r="P70" s="22"/>
     </row>
     <row r="71" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="26"/>
-      <c r="B71" s="26"/>
-      <c r="C71" s="30" t="s">
+      <c r="A71" s="22"/>
+      <c r="B71" s="22"/>
+      <c r="C71" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="D71" s="30"/>
-      <c r="E71" s="30"/>
-      <c r="F71" s="30"/>
-      <c r="G71" s="30"/>
-      <c r="H71" s="26"/>
-      <c r="I71" s="26"/>
-      <c r="J71" s="26"/>
-      <c r="K71" s="26"/>
-      <c r="L71" s="26"/>
-      <c r="M71" s="26"/>
-      <c r="N71" s="26"/>
-      <c r="O71" s="26"/>
-      <c r="P71" s="26"/>
+      <c r="D71" s="23"/>
+      <c r="E71" s="23"/>
+      <c r="F71" s="23"/>
+      <c r="G71" s="23"/>
+      <c r="H71" s="22"/>
+      <c r="I71" s="22"/>
+      <c r="J71" s="22"/>
+      <c r="K71" s="22"/>
+      <c r="L71" s="22"/>
+      <c r="M71" s="22"/>
+      <c r="N71" s="22"/>
+      <c r="O71" s="22"/>
+      <c r="P71" s="22"/>
     </row>
     <row r="72" spans="1:16" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="26"/>
-      <c r="B72" s="26"/>
-      <c r="C72" s="26"/>
-      <c r="D72" s="26"/>
-      <c r="E72" s="26"/>
-      <c r="F72" s="26"/>
-      <c r="G72" s="26"/>
-      <c r="H72" s="26"/>
-      <c r="I72" s="26"/>
-      <c r="J72" s="26"/>
-      <c r="K72" s="26"/>
-      <c r="L72" s="26"/>
-      <c r="M72" s="26"/>
-      <c r="N72" s="26"/>
-      <c r="O72" s="26"/>
-      <c r="P72" s="26"/>
+      <c r="A72" s="22"/>
+      <c r="B72" s="22"/>
+      <c r="C72" s="22"/>
+      <c r="D72" s="22"/>
+      <c r="E72" s="22"/>
+      <c r="F72" s="22"/>
+      <c r="G72" s="22"/>
+      <c r="H72" s="22"/>
+      <c r="I72" s="22"/>
+      <c r="J72" s="22"/>
+      <c r="K72" s="22"/>
+      <c r="L72" s="22"/>
+      <c r="M72" s="22"/>
+      <c r="N72" s="22"/>
+      <c r="O72" s="22"/>
+      <c r="P72" s="22"/>
     </row>
     <row r="73" spans="1:16" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="26"/>
-      <c r="B73" s="26"/>
-      <c r="C73" s="26"/>
-      <c r="D73" s="26"/>
-      <c r="E73" s="26"/>
-      <c r="F73" s="26"/>
-      <c r="G73" s="26"/>
-      <c r="H73" s="26"/>
-      <c r="I73" s="26"/>
-      <c r="J73" s="26"/>
-      <c r="K73" s="26"/>
-      <c r="L73" s="26"/>
-      <c r="M73" s="26"/>
-      <c r="N73" s="26"/>
-      <c r="O73" s="26"/>
-      <c r="P73" s="26"/>
+      <c r="A73" s="22"/>
+      <c r="B73" s="22"/>
+      <c r="C73" s="22"/>
+      <c r="D73" s="22"/>
+      <c r="E73" s="22"/>
+      <c r="F73" s="22"/>
+      <c r="G73" s="22"/>
+      <c r="H73" s="22"/>
+      <c r="I73" s="22"/>
+      <c r="J73" s="22"/>
+      <c r="K73" s="22"/>
+      <c r="L73" s="22"/>
+      <c r="M73" s="22"/>
+      <c r="N73" s="22"/>
+      <c r="O73" s="22"/>
+      <c r="P73" s="22"/>
     </row>
     <row r="74" spans="1:16" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="26"/>
-      <c r="B74" s="26"/>
-      <c r="C74" s="17" t="s">
+      <c r="A74" s="22"/>
+      <c r="B74" s="22"/>
+      <c r="C74" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="D74" s="28"/>
-      <c r="E74" s="28"/>
-      <c r="F74" s="28"/>
-      <c r="G74" s="26"/>
-      <c r="H74" s="26"/>
-      <c r="I74" s="26"/>
-      <c r="J74" s="26"/>
-      <c r="K74" s="26"/>
-      <c r="L74" s="26"/>
-      <c r="M74" s="34" t="s">
+      <c r="D74" s="27"/>
+      <c r="E74" s="27"/>
+      <c r="F74" s="27"/>
+      <c r="G74" s="22"/>
+      <c r="H74" s="22"/>
+      <c r="I74" s="22"/>
+      <c r="J74" s="22"/>
+      <c r="K74" s="22"/>
+      <c r="L74" s="22"/>
+      <c r="M74" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="N74" s="34"/>
-      <c r="O74" s="34"/>
-      <c r="P74" s="26"/>
+      <c r="N74" s="31"/>
+      <c r="O74" s="31"/>
+      <c r="P74" s="22"/>
     </row>
     <row r="75" spans="1:16" ht="13.7" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="26"/>
-      <c r="B75" s="26"/>
-      <c r="C75" s="26"/>
-      <c r="D75" s="26"/>
-      <c r="E75" s="26"/>
-      <c r="F75" s="26"/>
-      <c r="G75" s="26"/>
-      <c r="H75" s="26"/>
-      <c r="I75" s="26"/>
-      <c r="J75" s="26"/>
-      <c r="K75" s="26"/>
-      <c r="L75" s="26"/>
-      <c r="M75" s="26"/>
-      <c r="N75" s="26"/>
-      <c r="O75" s="26"/>
-      <c r="P75" s="26"/>
+      <c r="A75" s="22"/>
+      <c r="B75" s="22"/>
+      <c r="C75" s="22"/>
+      <c r="D75" s="22"/>
+      <c r="E75" s="22"/>
+      <c r="F75" s="22"/>
+      <c r="G75" s="22"/>
+      <c r="H75" s="22"/>
+      <c r="I75" s="22"/>
+      <c r="J75" s="22"/>
+      <c r="K75" s="22"/>
+      <c r="L75" s="22"/>
+      <c r="M75" s="22"/>
+      <c r="N75" s="22"/>
+      <c r="O75" s="22"/>
+      <c r="P75" s="22"/>
     </row>
     <row r="76" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B76" s="26"/>
-      <c r="C76" s="26"/>
-      <c r="D76" s="26"/>
-      <c r="E76" s="26"/>
-      <c r="F76" s="26"/>
-      <c r="G76" s="26"/>
-      <c r="H76" s="26"/>
-      <c r="I76" s="26"/>
-      <c r="J76" s="26"/>
-      <c r="K76" s="26"/>
-      <c r="L76" s="26"/>
-      <c r="M76" s="26"/>
-      <c r="N76" s="26"/>
-      <c r="O76" s="26"/>
-      <c r="P76" s="26"/>
+      <c r="B76" s="22"/>
+      <c r="C76" s="22"/>
+      <c r="D76" s="22"/>
+      <c r="E76" s="22"/>
+      <c r="F76" s="22"/>
+      <c r="G76" s="22"/>
+      <c r="H76" s="22"/>
+      <c r="I76" s="22"/>
+      <c r="J76" s="22"/>
+      <c r="K76" s="22"/>
+      <c r="L76" s="22"/>
+      <c r="M76" s="22"/>
+      <c r="N76" s="22"/>
+      <c r="O76" s="22"/>
+      <c r="P76" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="44">
+  <mergeCells count="46">
+    <mergeCell ref="C19:O19"/>
     <mergeCell ref="B75:P76"/>
     <mergeCell ref="K46:O50"/>
     <mergeCell ref="F48:J48"/>
@@ -2819,6 +2820,7 @@
     <mergeCell ref="C72:O73"/>
     <mergeCell ref="G74:L74"/>
     <mergeCell ref="M74:O74"/>
+    <mergeCell ref="H28:K28"/>
     <mergeCell ref="A1:P1"/>
     <mergeCell ref="A2:A75"/>
     <mergeCell ref="B2:B74"/>
@@ -2834,7 +2836,7 @@
     <mergeCell ref="F8:J8"/>
     <mergeCell ref="F10:J10"/>
     <mergeCell ref="F12:J12"/>
-    <mergeCell ref="C19:O19"/>
+    <mergeCell ref="K42:N42"/>
     <mergeCell ref="F34:J34"/>
     <mergeCell ref="F14:J14"/>
     <mergeCell ref="F20:J20"/>

</xml_diff>